<commit_message>
feat: add ia analisys
</commit_message>
<xml_diff>
--- a/paginas_encontradas.xlsx
+++ b/paginas_encontradas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,21 +425,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Serie</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Busqueda</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -446,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/tctelevision/p/DVORrImDeBs/?hl=af</t>
+          <t>https://www.instagram.com/p/DVOdiylkRc-/</t>
         </is>
       </c>
     </row>
@@ -463,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVOz-rogGXC/</t>
+          <t>https://www.instagram.com/tctelevision/p/DVORrImDeBs/?hl=af</t>
         </is>
       </c>
     </row>
@@ -480,7 +492,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVOSgCPkZjd/</t>
+          <t>https://www.instagram.com/p/DVOz-rogGXC/</t>
         </is>
       </c>
     </row>
@@ -497,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVOdiylkRc-/</t>
+          <t>https://www.instagram.com/p/DVOSgCPkZjd/</t>
         </is>
       </c>
     </row>
@@ -514,7 +526,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVMpuBIgEgM/</t>
+          <t>https://www.instagram.com/p/DJrtQepMxwi/</t>
         </is>
       </c>
     </row>
@@ -531,7 +543,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVMSBXUj67w/</t>
+          <t>https://www.instagram.com/p/DVMdRG4iYyX/</t>
         </is>
       </c>
     </row>
@@ -548,7 +560,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVMdRG4iYyX/</t>
+          <t>https://www.instagram.com/p/DT3FlgNDvHR/</t>
         </is>
       </c>
     </row>
@@ -565,7 +577,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUGzvSKCcYb/</t>
+          <t>https://www.instagram.com/p/DVMpuBIgEgM/</t>
         </is>
       </c>
     </row>
@@ -582,7 +594,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DSvPPdWkTwb/</t>
+          <t>https://www.instagram.com/p/DVPLEs_DodX/</t>
         </is>
       </c>
     </row>
@@ -599,7 +611,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUycL_tDOVR/</t>
+          <t>https://www.instagram.com/p/DUHgZlgEQG_/</t>
         </is>
       </c>
     </row>
@@ -633,7 +645,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DSyG11PF-B4/</t>
+          <t>https://www.instagram.com/p/DUFea54DG6x/</t>
         </is>
       </c>
     </row>
@@ -667,7 +679,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUGpQq-ET9_/</t>
+          <t>https://www.instagram.com/p/DSyG11PF-B4/</t>
         </is>
       </c>
     </row>
@@ -684,7 +696,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/reel/DUUbJnADa1G/</t>
+          <t>https://www.instagram.com/p/DUGpQq-ET9_/</t>
         </is>
       </c>
     </row>
@@ -735,7 +747,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUHgZlgEQG_/</t>
+          <t>https://www.instagram.com/reel/DUUbJnADa1G/</t>
         </is>
       </c>
     </row>
@@ -752,7 +764,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DTvwrTAEWuh/</t>
+          <t>https://www.instagram.com/p/DVST-buDMPt/</t>
         </is>
       </c>
     </row>
@@ -769,7 +781,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVST-buDMPt/</t>
+          <t>https://www.instagram.com/p/DSu-BlzEYzy/</t>
         </is>
       </c>
     </row>
@@ -786,7 +798,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUlEx1NjaYZ/</t>
+          <t>https://www.instagram.com/p/DUGyD-6j4ls/</t>
         </is>
       </c>
     </row>
@@ -803,7 +815,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUGyD-6j4ls/</t>
+          <t>https://www.instagram.com/p/DUlEx1NjaYZ/</t>
         </is>
       </c>
     </row>
@@ -820,7 +832,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUJH2TEDHrY/</t>
+          <t>https://www.instagram.com/p/DS5geZTDU8R/</t>
         </is>
       </c>
     </row>
@@ -837,7 +849,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DSu-BlzEYzy/</t>
+          <t>https://www.instagram.com/p/DUJH2TEDHrY/</t>
         </is>
       </c>
     </row>
@@ -854,7 +866,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUGftZ0jrum/</t>
+          <t>https://www.instagram.com/p/DUUOAlgj70E/</t>
         </is>
       </c>
     </row>
@@ -871,7 +883,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVPLEs_DodX/</t>
+          <t>https://www.instagram.com/p/DStkvG1DEUY/</t>
         </is>
       </c>
     </row>
@@ -888,7 +900,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DS5geZTDU8R/</t>
+          <t>https://www.instagram.com/p/DSvW5bUEsoO/</t>
         </is>
       </c>
     </row>
@@ -900,12 +912,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUUOAlgj70E/</t>
+          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/874579312061852/</t>
         </is>
       </c>
     </row>
@@ -917,12 +929,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/netflixlat/</t>
+          <t>https://www.facebook.com/cadenadelmarfm1065/videos/bridgerton-netflix-4%C2%AA-temporada-arrasa-y-vuelve-a-cautivar-al-p%C3%BAblico/2171927366915739/</t>
         </is>
       </c>
     </row>
@@ -934,12 +946,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVZEA-EjAVg/</t>
+          <t>https://www.facebook.com/ComfortUruguay/videos/una-nueva-pista-perfumada-llega-al-palacioel-secreto-est%C3%A1-a-punto-de-ser-revelad/1615445112706598/</t>
         </is>
       </c>
     </row>
@@ -956,7 +968,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/874579312061852/</t>
+          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/2378705162590136/</t>
         </is>
       </c>
     </row>
@@ -973,7 +985,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cadenadelmarfm1065/videos/bridgerton-netflix-4%C2%AA-temporada-arrasa-y-vuelve-a-cautivar-al-p%C3%BAblico/2171927366915739/</t>
+          <t>https://www.facebook.com/cartasaeliza/posts/ya-sabes-a-qu%C3%A9-hora-estar%C3%A1n-disponibles-los-nuevos-episodios-de-bridgerton-estad/1512664910859722/</t>
         </is>
       </c>
     </row>
@@ -990,7 +1002,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ComfortUruguay/videos/una-nueva-pista-perfumada-llega-al-palacioel-secreto-est%C3%A1-a-punto-de-ser-revelad/1615445112706598/</t>
+          <t>https://www.facebook.com/groups/769572330299468/posts/1762034177719940/</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1019,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/2378705162590136/</t>
+          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/1472684427721945/</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1036,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cartasaeliza/posts/ya-sabes-a-qu%C3%A9-hora-estar%C3%A1n-disponibles-los-nuevos-episodios-de-bridgerton-estad/1512664910859722/</t>
+          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/742416995394439/</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1053,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/769572330299468/posts/1762034177719940/</t>
+          <t>https://www.facebook.com/debateuruguaynoticias/posts/baile-de-m%C3%A1scaras-y-taylor-swift-se-estren%C3%B3-la-cuarta-temporada-de-los-bridgerto/877969608319032/</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1087,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/742416995394439/</t>
+          <t>https://www.facebook.com/NetflixArg/posts/este-es-el-evento-de-la-temporada-para-todos-los-fans-de-bridgertonel-9-de-febre/1330235185804528/</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1104,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/debateuruguaynoticias/posts/baile-de-m%C3%A1scaras-y-taylor-swift-se-estren%C3%B3-la-cuarta-temporada-de-los-bridgerto/877969608319032/</t>
+          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/1242972931091091/</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1121,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/1472684427721945/</t>
+          <t>https://www.facebook.com/elpaisuy/posts/de-bridgerton-a-la-odisea-de-nolan-y-hasta-una-pel%C3%ADcula-uruguaya-sobre-escritora/1232928072301948/</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1138,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/posts/este-es-el-evento-de-la-temporada-para-todos-los-fans-de-bridgertonel-9-de-febre/1330235185804528/</t>
+          <t>https://www.facebook.com/vovediariodigital/posts/-la-espera-de-los-fan%C3%A1ticos-de-bridgerton-llega-a-su-fin-finalmente-este-jueves-/1219537233704696/</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/posts/de-bridgerton-a-la-odisea-de-nolan-y-hasta-una-pel%C3%ADcula-uruguaya-sobre-escritora/1232928072301948/</t>
+          <t>https://www.facebook.com/RTSmedios/photos/espect%C3%A1culos-netflix-revel%C3%B3-t%C3%ADtulos-y-duraci%C3%B3n-de-los-primeros-episodios-de-la-c/1369331881873630/</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1172,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/vovediariodigital/posts/-la-espera-de-los-fan%C3%A1ticos-de-bridgerton-llega-a-su-fin-finalmente-este-jueves-/1219537233704696/</t>
+          <t>https://www.facebook.com/clarincom/posts/la-cuarta-temporada-debuta-este-29-de-enero-en-netflix-para-desentra%C3%B1ar-el-inici/1341408221354182/</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1189,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/clarincom/posts/la-cuarta-temporada-debuta-este-29-de-enero-en-netflix-para-desentra%C3%B1ar-el-inici/1341408221354182/</t>
+          <t>https://www.facebook.com/photo.php?fbid=1747795425302901&amp;id=299859170096541&amp;set=a.299860116763113</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1206,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/RTSmedios/photos/espect%C3%A1culos-netflix-revel%C3%B3-t%C3%ADtulos-y-duraci%C3%B3n-de-los-primeros-episodios-de-la-c/1369331881873630/</t>
+          <t>https://www.facebook.com/libreriaelvirreyuy/posts/tras-la-exitosa-saga-bridgerton-que-netflix-ha-convertido-en-una-serie-llega-la-/2858888594376833/</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1223,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ComfortUruguay/</t>
+          <t>https://www.facebook.com/ElObservadorUY/posts/bridgerton-fue-una-de-las-series-m%C3%A1s-vistas-en-netflix-el-verano-pasado-en-urugu/10159849239625842/?locale=hi_IN</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1240,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/libreriaelvirreyuy/posts/tras-la-exitosa-saga-bridgerton-que-netflix-ha-convertido-en-una-serie-llega-la-/2858888594376833/</t>
+          <t>https://www.facebook.com/elpaisuy/posts/netflix-revel%C3%B3-el-primer-adelanto-de-la-cuarta-temporada-de-bridgerton-y-confirm/1161703156091107/</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1257,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/photo.php?fbid=1747795425302901&amp;id=299859170096541&amp;set=a.299860116763113</t>
+          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/888088347102338/</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1274,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/posts/netflix-revel%C3%B3-el-primer-adelanto-de-la-cuarta-temporada-de-bridgerton-y-confirm/1161703156091107/</t>
+          <t>https://www.facebook.com/tvshowuy/posts/m%C3%A1s-oscura-y-melanc%C3%B3lica-detalles-de-la-temporada-4-de-bridgerton-y-cu%C3%A1ndo-se-es/1585824876351505/</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1291,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ElObservadorUY/posts/bridgerton-fue-una-de-las-series-m%C3%A1s-vistas-en-netflix-el-verano-pasado-en-urugu/10159849239625842/?locale=hi_IN</t>
+          <t>https://www.facebook.com/ComfortUruguay/videos/las-flores-desaparecieron-de-manera-misteriosa-el-secreto-m%C3%A1s-perfumado-podr%C3%A1-se/25344967681849805/</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1308,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ComfortUruguay/videos/las-flores-desaparecieron-de-manera-misteriosa-el-secreto-m%C3%A1s-perfumado-podr%C3%A1-se/25344967681849805/</t>
+          <t>https://www.facebook.com/perfilcom/posts/a-qu%C3%A9-hora-se-estren%C3%B3-en-netflix-la-segunda-parte-de-bridgerton-4-en-argentina/1353904796770185/</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1325,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/863898726412695/</t>
+          <t>https://www.facebook.com/ComfortUruguay/videos/las-flores-desaparecieron-de-manera-misteriosa-el-secreto-m%C3%A1s-perfumado-podr%C3%A1-se/893079166830234/</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1342,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/888088347102338/</t>
+          <t>https://www.facebook.com/photo.php?fbid=1140471294916091&amp;set=a.421318166831411&amp;id=100068596927356</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1359,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/tvshowuy/posts/m%C3%A1s-oscura-y-melanc%C3%B3lica-detalles-de-la-temporada-4-de-bridgerton-y-cu%C3%A1ndo-se-es/1585824876351505/</t>
+          <t>https://www.facebook.com/lannistercomics/posts/atenci%C3%B3n-amantes-de-bridgerton-disponible-la-colecci%C3%B3n-completa-se-estreno-la-2d/5591876737525968/</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1376,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/perfilcom/posts/a-qu%C3%A9-hora-se-estren%C3%B3-en-netflix-la-segunda-parte-de-bridgerton-4-en-argentina/1353904796770185/</t>
+          <t>https://www.facebook.com/ComfortUruguay/</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1393,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ComfortUruguay/videos/las-flores-desaparecieron-de-manera-misteriosa-el-secreto-m%C3%A1s-perfumado-podr%C3%A1-se/893079166830234/</t>
+          <t>https://www.facebook.com/lannistercomics/posts/saga-de-g%C3%A9nero-romance-hist%C3%B3rico-los-bridgerton-escrita-por-julia-quinn-y-public/4591684954211823/</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1410,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-3-parte-2/448650128016965/</t>
+          <t>https://www.facebook.com/groups/769572330299468/posts/1727394321183926/</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1427,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/posts/netflix-asegura-que-bridgerton-es-la-serie-m%C3%A1s-vista-de-toda-su-historia-la-prod/10160662759376754/</t>
+          <t>https://www.facebook.com/EmbajadaBritanicaMontevideo/posts/-ya-vieron-la-nueva-serie-de-netflix-queen-charlotte-si-bien-la-serie-ocurre-en-/577169867833684/</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1461,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/769572330299468/posts/1727394321183926/</t>
+          <t>https://www.facebook.com/elpaisuy/posts/netflix-asegura-que-bridgerton-es-la-serie-m%C3%A1s-vista-de-toda-su-historia-la-prod/10160662759376754/</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1478,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/photos/netflix-revel%C3%B3-el-primer-adelanto-de-la-cuarta-temporada-de-bridgerton-y-confirm/1161703139424442/</t>
+          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-3-parte-2/448650128016965/</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1495,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/redessocialesarg/videos/un-paseo-estilo-bridgerton-gratis-en-buenos-aires-s%C3%AD-est%C3%A1-pasandonetflix-organiz/926751779827211/</t>
+          <t>https://www.facebook.com/elpaisuy/photos/netflix-revel%C3%B3-el-primer-adelanto-de-la-cuarta-temporada-de-bridgerton-y-confirm/1161703139424442/</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1512,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/posts/netflix-asegura-que-bridgerton-es-la-serie-m%C3%A1s-vista-de-toda-su-historia-la-prod/10160660939456754/</t>
+          <t>https://www.facebook.com/BridgertonLatinoamerica/posts/ay-ben-te-mmste-%EF%B8%8Fbridgerton-bridgertonnetflix-benedictbridgerton-netflix/1345480020959147/</t>
         </is>
       </c>
     </row>
@@ -1512,12 +1524,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7600424191522786573</t>
+          <t>https://www.facebook.com/redessocialesarg/videos/un-paseo-estilo-bridgerton-gratis-en-buenos-aires-s%C3%AD-est%C3%A1-pasandonetflix-organiz/926751779827211/</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1541,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@milakate1999/video/7606732930806729991</t>
+          <t>https://www.facebook.com/elpaisuy/posts/netflix-asegura-que-bridgerton-es-la-serie-m%C3%A1s-vista-de-toda-su-historia-la-prod/10160660939456754/</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1563,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixlat/video/7593055754735865096</t>
+          <t>https://www.tiktok.com/@chenetflix/video/7600424191522786573</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1580,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixlat/video/7602268274629397776</t>
+          <t>https://www.tiktok.com/@milakate1999/video/7606732930806729991</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1597,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7595703870014131469</t>
+          <t>https://www.tiktok.com/@netflixlat/video/7593055754735865096</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1614,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7609844795061652749</t>
+          <t>https://www.tiktok.com/@netflixlat/video/7602268274629397776</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1631,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixes/video/7600447840447581462</t>
+          <t>https://www.tiktok.com/@chenetflix/video/7595703870014131469</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1648,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7595649570139344142</t>
+          <t>https://www.tiktok.com/@chenetflix/video/7609844795061652749</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1665,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@eugepuche/video/7611298973923495176</t>
+          <t>https://www.tiktok.com/@netflixes/video/7600447840447581462</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1682,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@pijama.surf/video/7600861625373035796</t>
+          <t>https://www.tiktok.com/@chenetflix/video/7595649570139344142</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1699,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/discover/cuando-sale-bridgerton-4-en-argentina</t>
+          <t>https://www.tiktok.com/@eugepuche/video/7611298973923495176</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1716,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixlat/video/7369335819200449793</t>
+          <t>https://www.tiktok.com/discover/cuando-sale-bridgerton-4-en-argentina</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1733,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixlat/video/7603930655117872404</t>
+          <t>https://www.tiktok.com/@netflixlat/video/7369335819200449793</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1750,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7598326974951607565</t>
+          <t>https://www.tiktok.com/@cpher_art/video/7609546888773127445</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1767,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7601155903466851598</t>
+          <t>https://www.tiktok.com/@netflixlat/video/7603930655117872404</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1801,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cpher_art/video/7609546888773127445</t>
+          <t>https://www.tiktok.com/@marcoseyo/video/7601633663150722311</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1835,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@apasionadosxviajar/video/7609550112158764309</t>
+          <t>https://www.tiktok.com/@chulaenlaluna/video/7600849139949112583</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1852,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@marcoseyo/video/7601633663150722311</t>
+          <t>https://www.tiktok.com/@onlinemami_/video/7610200734360964360</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1869,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chulaenlaluna/video/7600849139949112583</t>
+          <t>https://www.tiktok.com/@chenetflix/video/7598326974951607565</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1886,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7358085398805007658</t>
+          <t>https://www.tiktok.com/@netflixes/video/7367679551809277216</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1903,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mariaspeaksenglish/video/7369691983713094945</t>
+          <t>https://www.tiktok.com/@chenetflix/video/7358085398805007658</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1920,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixes/video/7367679551809277216</t>
+          <t>https://www.tiktok.com/@alewkd/video/7367172113842654470</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1937,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@alewkd/video/7367172113842654470</t>
+          <t>https://www.tiktok.com/@adriianabad99/video/7601432071604702487</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1954,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/discover/bridgerton-argentina-victoria-resco</t>
+          <t>https://www.tiktok.com/@chenetflix/video/7606441973901233422</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1971,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7606441973901233422</t>
+          <t>https://www.tiktok.com/@hoyestaparaleer/video/7370405528113057029</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1988,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@adriianabad99/video/7601432071604702487</t>
+          <t>https://www.tiktok.com/@onlinemami_/video/7595735741922168082</t>
         </is>
       </c>
     </row>
@@ -1988,12 +2000,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@suny.jks/video/7603162089301003528</t>
+          <t>https://www.youtube.com/channel/UC5ZiUaIJ2b5dYBYGf5iEUrA</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2056,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=UsAEQwTAuH0</t>
+          <t>https://m.youtube.com/@LADSpanishTV-8386x/videos?view=0&amp;sort=dd&amp;shelf_id=2</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2073,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/hashtag/staircasescene</t>
+          <t>https://www.youtube.com/watch?v=kMXQlA14JBQ</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2090,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/c/aragondigital/channels</t>
+          <t>https://www.youtube.com/watch?v=UsAEQwTAuH0</t>
         </is>
       </c>
     </row>
@@ -2090,12 +2102,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
+          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=kMXQlA14JBQ</t>
+          <t>https://x.com/DebateUruguay_/status/2017275931405258915</t>
         </is>
       </c>
     </row>
@@ -2107,12 +2119,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
+          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://m.youtube.com/@LADSpanishTV-8386x/videos?view=0&amp;sort=dd&amp;shelf_id=2</t>
+          <t>https://x.com/agusc4brera</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2141,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://x.com/DebateUruguay_/status/2017275931405258915</t>
+          <t>https://x.com/elpaisuy/status/1344705160375894019</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2158,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://x.com/agusc4brera</t>
+          <t>https://x.com/vicky_oyhenart</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2175,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://x.com/elpaisuy/status/1344705160375894019</t>
+          <t>https://x.com/proximapaginaok</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2192,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://x.com/vicky_oyhenart</t>
+          <t>https://x.com/XimeCoonX</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2209,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>https://x.com/proximapaginaok</t>
+          <t>https://x.com/nadia2abi</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2226,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://x.com/XimeCoonX</t>
+          <t>https://x.com/karenreiscach</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2243,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>https://x.com/nadia2abi</t>
+          <t>https://x.com/lizkocacomert</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2260,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>https://x.com/karenreiscach</t>
+          <t>https://x.com/NBonin/status/1797486263148396771</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2277,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://x.com/lizkocacomert</t>
+          <t>https://x.com/cruzher30</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2294,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://x.com/NBonin/status/1797486263148396771</t>
+          <t>https://x.com/__lavenderhaze</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2311,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>https://x.com/arissanchezzz</t>
+          <t>https://x.com/anto_z31</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2328,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>https://x.com/__lavenderhaze</t>
+          <t>https://x.com/itchytaglitter?lang=da</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2345,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>https://x.com/anto_z31</t>
+          <t>https://x.com/laboraton</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2379,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://x.com/laboraton</t>
+          <t>https://x.com/mpazperalta</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2396,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://x.com/mpazperalta</t>
+          <t>https://x.com/Gala0374</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2430,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://x.com/Gala0374</t>
+          <t>https://x.com/puig_vero</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2447,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://x.com/puig_vero</t>
+          <t>https://x.com/arissanchezzz</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2481,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>https://x.com/newslinereport</t>
+          <t>https://x.com/lys_12</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2498,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>https://x.com/lecturasdeannie</t>
+          <t>https://x.com/florenciaamorin</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2515,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>https://x.com/MaugeGarcia</t>
+          <t>https://x.com/ddl_sophie97</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2532,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>https://x.com/florenciaamorin</t>
+          <t>https://x.com/lecturasdeannie</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2549,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>https://x.com/ddl_sophie97</t>
+          <t>https://x.com/Aurorakillian30</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2566,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>https://x.com/lys_12</t>
+          <t>https://x.com/Manuu_CYfan</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2583,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>https://x.com/Aurorakillian30</t>
+          <t>https://x.com/nazagaggero</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2600,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>https://x.com/Manuu_CYfan</t>
+          <t>https://x.com/newslinereport</t>
         </is>
       </c>
     </row>
@@ -2605,41 +2617,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>https://x.com/search?lang=es&amp;q=Sigue%20plataforma%20DUTT%20comentarios%202026%20usuarios%20reales.uns</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>Bridgerton</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>https://x.com/nazagaggero</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Bridgerton</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>https://x.com/tartancrepes</t>
+          <t>https://x.com/IvanQuiroga_Ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement ia analysis with groq
</commit_message>
<xml_diff>
--- a/paginas_encontradas.xlsx
+++ b/paginas_encontradas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,2176 +448,2278 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVOdiylkRc-/</t>
+          <t>https://www.instagram.com/reel/DUisvo-jChN/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/tctelevision/p/DVORrImDeBs/?hl=af</t>
+          <t>https://www.instagram.com/reel/DKabsuRy6Ab/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVOz-rogGXC/</t>
+          <t>https://www.instagram.com/reel/DTVueIGCYHM/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVOSgCPkZjd/</t>
+          <t>https://www.instagram.com/p/DTVjL6VDnQL/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJrtQepMxwi/</t>
+          <t>https://www.instagram.com/p/DUoXh9pjysE/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVMdRG4iYyX/</t>
+          <t>https://www.instagram.com/p/DTjLRtKjbcx/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DT3FlgNDvHR/</t>
+          <t>https://www.instagram.com/p/DTv7ZRCkRc4/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVMpuBIgEgM/</t>
+          <t>https://www.instagram.com/p/DTZN-s3jNWz/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVPLEs_DodX/</t>
+          <t>https://www.instagram.com/p/DQrfmq3jcGs/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUHgZlgEQG_/</t>
+          <t>https://www.instagram.com/p/DTjno7ZjhBU/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUPD4U9Dj3H/</t>
+          <t>https://www.instagram.com/p/DS5nJoLEVrj/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUFea54DG6x/</t>
+          <t>https://www.instagram.com/p/DUEErQakZE5/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/reel/DVE-d1EibtV/</t>
+          <t>https://www.instagram.com/p/DUm3vtogEoX/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DSyG11PF-B4/</t>
+          <t>https://www.instagram.com/p/DTvXfDcgW7i/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUGpQq-ET9_/</t>
+          <t>https://www.instagram.com/p/DS2nnk4kb4T/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVPsr7HjUQR/</t>
+          <t>https://www.instagram.com/p/DTjUEEej23q/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUJlHkvkbJu/</t>
+          <t>https://www.instagram.com/p/DUgSJBMkdsU/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/reel/DUUbJnADa1G/</t>
+          <t>https://www.instagram.com/p/DUohKr_D-fH/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVST-buDMPt/</t>
+          <t>https://www.instagram.com/reel/DRf7Df0iPUS/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DSu-BlzEYzy/</t>
+          <t>https://www.instagram.com/reel/DTbqxbKAKZr/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUGyD-6j4ls/</t>
+          <t>https://www.instagram.com/p/DTlWekdkab5/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUlEx1NjaYZ/</t>
+          <t>https://www.instagram.com/p/DTLNyLXitno/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DS5geZTDU8R/</t>
+          <t>https://www.instagram.com/p/DSypREHjYfB/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUJH2TEDHrY/</t>
+          <t>https://www.instagram.com/p/DTjNVQSDQJF/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUUOAlgj70E/</t>
+          <t>https://www.instagram.com/p/DT_mvOClUuJ/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DStkvG1DEUY/</t>
+          <t>https://www.instagram.com/p/DTk_AH-jb2K/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:instagram.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DSvW5bUEsoO/</t>
+          <t>https://www.instagram.com/p/DTg48PPiLr5/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/874579312061852/</t>
+          <t>https://www.instagram.com/p/DTtDGgaiEKC/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cadenadelmarfm1065/videos/bridgerton-netflix-4%C2%AA-temporada-arrasa-y-vuelve-a-cautivar-al-p%C3%BAblico/2171927366915739/</t>
+          <t>https://www.instagram.com/p/DTvKjQUjc0U/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ComfortUruguay/videos/una-nueva-pista-perfumada-llega-al-palacioel-secreto-est%C3%A1-a-punto-de-ser-revelad/1615445112706598/</t>
+          <t>https://www.instagram.com/p/DTgj_FSicOu/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:instagram.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/2378705162590136/</t>
+          <t>https://www.instagram.com/reel/DTP8FBDjl5B/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cartasaeliza/posts/ya-sabes-a-qu%C3%A9-hora-estar%C3%A1n-disponibles-los-nuevos-episodios-de-bridgerton-estad/1512664910859722/</t>
+          <t>https://www.facebook.com/61566493452345/posts/la-reina-del-flow-3-estreno-oficial-netflix-y-que-dia-salver-m%C3%A1s/122177119484549781/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/769572330299468/posts/1762034177719940/</t>
+          <t>https://www.facebook.com/CaracolTVIntl/posts/el-fen%C3%B3meno-mundial-regresala-reina-del-flow-3-ya-est%C3%A1-disponible-con-sus-primer/1494031882731003/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/1472684427721945/</t>
+          <t>https://www.facebook.com/61566493452345/posts/la-reina-del-flow-3-estreno-oficial-en-netflix-y-avancver-m%C3%A1s/122165786636549781/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/742416995394439/</t>
+          <t>https://www.facebook.com/CaracolTVIntl/posts/el-flow-no-para-lareinadelflow3-se-mantiene-en-el-top-10-de-europa-y-am%C3%A9rica-lis/1520423473425177/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/debateuruguaynoticias/posts/baile-de-m%C3%A1scaras-y-taylor-swift-se-estren%C3%B3-la-cuarta-temporada-de-los-bridgerto/877969608319032/</t>
+          <t>https://www.facebook.com/cacorali/posts/el-14-de-enero-de-2026-se-estrena-en-netflix-la-reina-del-flow-3/1254500930067645/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/887334047385646/</t>
+          <t>https://www.facebook.com/LOS40Colombia/posts/te-contamos-httpslos40comco20260115cuando-se-estrenan-los-nuevos-episodios-de-la/944258211597340/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/posts/este-es-el-evento-de-la-temporada-para-todos-los-fans-de-bridgertonel-9-de-febre/1330235185804528/</t>
+          <t>https://www.facebook.com/CaracolTVIntl/photos/el-flow-se-hace-sentir-en-todo-el-mundo-lareinadelflow3-est%C3%A1-presente-desde-el-d/1495420059258852/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/1242972931091091/</t>
+          <t>https://www.facebook.com/charlyflowof9/posts/faltan-3-d%C3%ADas-para-el-estreno-en-netflix-%EF%B8%8F-lareinadelflow/1211012641124597/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/posts/de-bridgerton-a-la-odisea-de-nolan-y-hasta-una-pel%C3%ADcula-uruguaya-sobre-escritora/1232928072301948/</t>
+          <t>https://www.facebook.com/elpaisuy/posts/la-reina-del-flow-cinco-claves-para-un-%C3%A9xito-de-netflix-a-puro-reggaeton-y-traic/10161565616471754/?locale=ms_MY</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/vovediariodigital/posts/-la-espera-de-los-fan%C3%A1ticos-de-bridgerton-llega-a-su-fin-finalmente-este-jueves-/1219537233704696/</t>
+          <t>https://www.facebook.com/groups/1561085184508241/posts/1899323187351104/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/RTSmedios/photos/espect%C3%A1culos-netflix-revel%C3%B3-t%C3%ADtulos-y-duraci%C3%B3n-de-los-primeros-episodios-de-la-c/1369331881873630/</t>
+          <t>https://www.facebook.com/61566493452345/posts/la-reina-del-flow-3-cap%C3%ADtulo-1-el-regreso-de-charly-y-suver-m%C3%A1s/122191883432549781/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/clarincom/posts/la-cuarta-temporada-debuta-este-29-de-enero-en-netflix-para-desentra%C3%B1ar-el-inici/1341408221354182/</t>
+          <t>https://www.facebook.com/CaracolTVIntl/photos/el-flow-no-para-lareinadelflow3-se-mantiene-en-el-top-10-de-europa-y-am%C3%A9rica-lis/1520423456758512/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/photo.php?fbid=1747795425302901&amp;id=299859170096541&amp;set=a.299860116763113</t>
+          <t>https://www.facebook.com/107733597773339/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/libreriaelvirreyuy/posts/tras-la-exitosa-saga-bridgerton-que-netflix-ha-convertido-en-una-serie-llega-la-/2858888594376833/</t>
+          <t>https://www.facebook.com/groups/578566984666491/posts/897204959469357/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ElObservadorUY/posts/bridgerton-fue-una-de-las-series-m%C3%A1s-vistas-en-netflix-el-verano-pasado-en-urugu/10159849239625842/?locale=hi_IN</t>
+          <t>https://www.facebook.com/CaracolTVIntl/posts/yeimy-montoya-est%C3%A1-de-regreso-y-va-por-todo-la-temporada-3-de-la-reina-del-flow-/1494322319368626/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/posts/netflix-revel%C3%B3-el-primer-adelanto-de-la-cuarta-temporada-de-bridgerton-y-confirm/1161703156091107/</t>
+          <t>https://www.facebook.com/CaracolTVIntl/posts/d%C3%ADa-1-el-a%C3%B1o-empieza-con-flow-conoce-todo-sobre-el-fen%C3%B3meno-mundial-en-content-a/1499538222180369/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-netflix/888088347102338/</t>
+          <t>https://www.facebook.com/groups/320209418102813/posts/9890587694398223/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/tvshowuy/posts/m%C3%A1s-oscura-y-melanc%C3%B3lica-detalles-de-la-temporada-4-de-bridgerton-y-cu%C3%A1ndo-se-es/1585824876351505/</t>
+          <t>https://www.facebook.com/61566493452345/photos/la-reina-del-flow-3-avance-cap%C3%ADtulo-41-yeimver-m%C3%A1s/122203698758549781/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ComfortUruguay/videos/las-flores-desaparecieron-de-manera-misteriosa-el-secreto-m%C3%A1s-perfumado-podr%C3%A1-se/25344967681849805/</t>
+          <t>https://www.facebook.com/61566804145750/posts/la-reina-del-flow-3-cap%C3%ADtulo-1-fecha-de-estreno-cu%C3%A1ndo-salever-m%C3%A1s/122175081392560138/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/perfilcom/posts/a-qu%C3%A9-hora-se-estren%C3%B3-en-netflix-la-segunda-parte-de-bridgerton-4-en-argentina/1353904796770185/</t>
+          <t>https://www.facebook.com/cacorali/posts/hola-nuestra-gente-linda-y-bella-gracias-por-vernos-por-tanto-cari%C3%B1o-y-aprecio-p/1266496085534796/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ComfortUruguay/videos/las-flores-desaparecieron-de-manera-misteriosa-el-secreto-m%C3%A1s-perfumado-podr%C3%A1-se/893079166830234/</t>
+          <t>https://www.facebook.com/magacin247/posts/la-reina-del-flow-3-cap%C3%ADtulo-20-final-ya-est%C3%A1-en-netflixel-esperado-episodio-fin/1239260678401965/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/photo.php?fbid=1140471294916091&amp;set=a.421318166831411&amp;id=100068596927356</t>
+          <t>https://www.facebook.com/100091764826058/posts/only-four-days-to-go-until-yeimy-and-charly-light-up-our-screens-once-again-lare/829154900153330/</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/lannistercomics/posts/atenci%C3%B3n-amantes-de-bridgerton-disponible-la-colecci%C3%B3n-completa-se-estreno-la-2d/5591876737525968/</t>
+          <t>https://www.facebook.com/elpaisuy/posts/estrella-de-una-de-las-series-latinas-m%C3%A1s-vistas-en-la-historia-de-netflix-viene/832496892345070/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ComfortUruguay/</t>
+          <t>https://www.facebook.com/61566493452345/posts/la-reina-del-flow-3-sky-se-enamora-de-charlver-m%C3%A1s/122192511440549781/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/lannistercomics/posts/saga-de-g%C3%A9nero-romance-hist%C3%B3rico-los-bridgerton-escrita-por-julia-quinn-y-public/4591684954211823/</t>
+          <t>https://www.facebook.com/Rapzadbarrio/posts/cuando-llegu%C3%A9-a-la-reina-del-flow-no-tra%C3%ADa-discursos-ni-promesas-tra%C3%ADa-tres-cap%C3%AD/1404652861030203/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/769572330299468/posts/1727394321183926/</t>
+          <t>https://www.facebook.com/Rapzadbarrio/posts/con-el-coraz%C3%B3n-lleno-de-felicidad-le-digo-a-todos-los-seguidores-de-la-reina-del/1411391973689625/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EmbajadaBritanicaMontevideo/posts/-ya-vieron-la-nueva-serie-de-netflix-queen-charlotte-si-bien-la-serie-ocurre-en-/577169867833684/</t>
+          <t>https://www.facebook.com/p/fanscarocaliuy-100064626826536/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-3-parte-2/464109322937601/</t>
+          <t>https://www.facebook.com/photo.php?fbid=1233121625538909&amp;set=a.419824346868645&amp;id=100065232504372</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/posts/netflix-asegura-que-bridgerton-es-la-serie-m%C3%A1s-vista-de-toda-su-historia-la-prod/10160662759376754/</t>
+          <t>https://www.facebook.com/61566493452345/posts/la-reina-del-flow-3-cap%C3%ADtulo-2-la-hija-de-los-reyes-del-flver-m%C3%A1s/122165789336549781/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:facebook.com</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/NetflixArg/videos/bridgerton-3-parte-2/448650128016965/</t>
+          <t>https://www.facebook.com/carocalimx1/posts/deja-tu-opini%C3%B3n-si-anticipas-con-entusiasmo-la-llegada-del-13-de-enero-de-2026-p/863246672966629/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/photos/netflix-revel%C3%B3-el-primer-adelanto-de-la-cuarta-temporada-de-bridgerton-y-confirm/1161703139424442/</t>
+          <t>https://www.tiktok.com/@_lorenaamartiin_/video/7586754744983588118</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/BridgertonLatinoamerica/posts/ay-ben-te-mmste-%EF%B8%8Fbridgerton-bridgertonnetflix-benedictbridgerton-netflix/1345480020959147/</t>
+          <t>https://www.tiktok.com/@karolinesita/video/7603443290523880726</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/redessocialesarg/videos/un-paseo-estilo-bridgerton-gratis-en-buenos-aires-s%C3%AD-est%C3%A1-pasandonetflix-organiz/926751779827211/</t>
+          <t>https://www.tiktok.com/@kiarareina16/video/7601552624520940822</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:facebook.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/elpaisuy/posts/netflix-asegura-que-bridgerton-es-la-serie-m%C3%A1s-vista-de-toda-su-historia-la-prod/10160660939456754/</t>
+          <t>https://www.tiktok.com/@ceciliafernandez222/video/7596311763830738188</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7600424191522786573</t>
+          <t>https://www.tiktok.com/discover/cuando-se-estrena-la-reina-del-flow-3-en-netflix-en-uruguay</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@milakate1999/video/7606732930806729991</t>
+          <t>https://www.tiktok.com/discover/cuando-se-estrena-la-reina-del-flow-3-en-uruguay</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixlat/video/7593055754735865096</t>
+          <t>https://www.tiktok.com/@carlos1torres1chile/video/7448310383439400198</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixlat/video/7602268274629397776</t>
+          <t>https://www.tiktok.com/discover/cu%C3%A1ndo-sale-la-reina-del-flow-en-uruguay</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7595703870014131469</t>
+          <t>https://www.tiktok.com/discover/la-reina-del-flow-3-estreno-fecha-2025-en-netflix</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7609844795061652749</t>
+          <t>https://www.tiktok.com/@aura.series/photo/7595330636265671944?lang=tr-TR</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixes/video/7600447840447581462</t>
+          <t>https://www.tiktok.com/@caracoltv/video/7594237575699729671</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7595649570139344142</t>
+          <t>https://www.tiktok.com/@carlos1torres1chile/video/7454264991202544901</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@eugepuche/video/7611298973923495176</t>
+          <t>https://www.tiktok.com/discover/cuando-estrena-la-reina-del-flow-3-en-magi</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/discover/cuando-sale-bridgerton-4-en-argentina</t>
+          <t>https://www.tiktok.com/discover/netflix-confirma-la-reina-del-flow-3-vienen-a-costa-rica</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixlat/video/7369335819200449793</t>
+          <t>https://www.tiktok.com/discover/ya-sali%C3%B3-la-reina-del-flow-en-netflix-de-brasil</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cpher_art/video/7609546888773127445</t>
+          <t>https://www.tiktok.com/discover/cuando-sale-la-reina-del-flow-3-en-uruguay</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixlat/video/7603930655117872404</t>
+          <t>https://www.tiktok.com/@caracoltvintl/video/7593403712970919175</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@topic.media/video/7394894841613683973</t>
+          <t>https://www.tiktok.com/@janibejaranonews/video/7592820334475152660</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@marcoseyo/video/7601633663150722311</t>
+          <t>https://www.tiktok.com/discover/a-qu%C3%A9-hora-se-estrena-la-reina-del-flow-en-netflix</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7610098651112705294</t>
+          <t>https://www.tiktok.com/discover/cuando-sale-la-reina-del-flow-3-de-2025</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chulaenlaluna/video/7600849139949112583</t>
+          <t>https://www.tiktok.com/discover/cuando-se-estrena-la-reina-del-flow-3-en-ecuador</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@onlinemami_/video/7610200734360964360</t>
+          <t>https://www.tiktok.com/@carlostorresfanpage/video/7573028963681881366</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7598326974951607565</t>
+          <t>https://www.tiktok.com/discover/cuando-sale-la-3-temporada-de-la-reina-del-flow-en-uruguay</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@netflixes/video/7367679551809277216</t>
+          <t>https://www.tiktok.com/discover/la-reina-del-flow-3-ya-esta-en-netflix</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7358085398805007658</t>
+          <t>https://www.tiktok.com/@noticiascaracol/video/7594960668655226123</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@alewkd/video/7367172113842654470</t>
+          <t>https://www.tiktok.com/@aleperu_/video/7595177348345924871</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@adriianabad99/video/7601432071604702487</t>
+          <t>https://www.tiktok.com/discover/cuando-se-estrena-la-reina-del-flow-3-en-argentina-netflix</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chenetflix/video/7606441973901233422</t>
+          <t>https://www.tiktok.com/discover/cuando-sale-en-netflix-la-reina-de-flow</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hoyestaparaleer/video/7370405528113057029</t>
+          <t>https://www.tiktok.com/@charleimy.fr/video/7586830899900189974</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:tiktok.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@onlinemami_/video/7595735741922168082</t>
+          <t>https://www.tiktok.com/discover/a-que-hora-sale-la-reina-del-flow-3-en-netflix</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/channel/UC5ZiUaIJ2b5dYBYGf5iEUrA</t>
+          <t>https://www.tiktok.com/discover/como-encuentro-en-netflix-los-capitulos-de-la-reina-del-flow</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=IAqV-7F-brg</t>
+          <t>https://www.tiktok.com/@aura.series/photo/7595330636265671944?lang=hu-HU</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:tiktok.com</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=0NSWp5airvo</t>
+          <t>https://www.tiktok.com/@la.reina.del.flowoficial/video/7280343680286805254</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://m.youtube.com/@LADSpanishTV-8386x/videos?view=0&amp;sort=dd&amp;shelf_id=2</t>
+          <t>https://www.youtube.com/watch?v=hQRTiLbQo8I</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=kMXQlA14JBQ</t>
+          <t>https://www.youtube.com/watch?v=941-adg1sbc</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:youtube.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=UsAEQwTAuH0</t>
+          <t>https://www.youtube.com/watch?v=8_HjNe13fTA</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://x.com/DebateUruguay_/status/2017275931405258915</t>
+          <t>https://www.youtube.com/playlist?list=PLL485KLzcXN5JWXwILq4HkDIkEgqVVTJI</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://x.com/agusc4brera</t>
+          <t>https://m.youtube.com/watch?v=MB_9VOgsQCo</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://x.com/elpaisuy/status/1344705160375894019</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://x.com/vicky_oyhenart</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=0</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://x.com/proximapaginaok</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=125</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://x.com/XimeCoonX</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=173</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>https://x.com/nadia2abi</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=410</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://x.com/karenreiscach</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=497</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>https://x.com/lizkocacomert</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=861</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>https://x.com/NBonin/status/1797486263148396771</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=1060</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://x.com/cruzher30</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=1200</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://x.com/__lavenderhaze</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=1303</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>https://x.com/anto_z31</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=1450</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>https://x.com/itchytaglitter?lang=da</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=1740</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>https://x.com/laboraton</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=1944</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>https://x.com/feer__olvv</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=2043</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://x.com/mpazperalta</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=2310</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://x.com/Gala0374</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=2550</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://x.com/Jotadangz</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=2714</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://x.com/puig_vero</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=3035</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://x.com/arissanchezzz</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=3235</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>https://x.com/search?q=%23OCCH%C4%B0AM%C4%B0N&amp;src=typed_query</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=3253</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>https://x.com/lys_12</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=3497</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>https://x.com/florenciaamorin</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=3787</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>https://x.com/ddl_sophie97</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=3951</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>https://x.com/lecturasdeannie</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=4208</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>https://x.com/Aurorakillian30</t>
+          <t>https://www.youtube.com/watch?v=d-HB1_e67hw&amp;t=4260</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>https://x.com/Manuu_CYfan</t>
+          <t>https://www.youtube.com/watch?v=Ga_WAsfzzAA</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>https://x.com/nazagaggero</t>
+          <t>https://m.youtube.com/@jrukc</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>https://x.com/newslinereport</t>
+          <t>https://www.youtube.com/watch?v=Bu7VDlvBvpk</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Bridgerton</t>
+          <t>la reina del flow</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>"Bridgerton" Netflix Uruguay site:x.com</t>
+          <t>"la reina del flow" Netflix Uruguay site:youtube.com</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>https://x.com/IvanQuiroga_Ok</t>
+          <t>https://www.youtube.com/watch?v=rYVTrL8FCao</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>la reina del flow</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>"la reina del flow" Netflix Uruguay site:x.com</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://x.com/prensario</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>la reina del flow</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>"la reina del flow" Netflix Uruguay site:x.com</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://x.com/miguelsmirnoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>la reina del flow</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>"la reina del flow" Netflix Uruguay site:x.com</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://x.com/VickyFraRu</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>la reina del flow</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>"la reina del flow" Netflix Uruguay site:x.com</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://x.com/yuryosma?lang=ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>la reina del flow</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>"la reina del flow" Netflix Uruguay site:x.com</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://x.com/arissanchezzz</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>la reina del flow</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>"la reina del flow" Netflix Uruguay site:x.com</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://x.com/Maaru_Caano</t>
         </is>
       </c>
     </row>

</xml_diff>